<commit_message>
Update tables & plots
</commit_message>
<xml_diff>
--- a/Tables/AAR_harris.xlsx
+++ b/Tables/AAR_harris.xlsx
@@ -486,25 +486,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.2544048509142</v>
+        <v>1.107004786128738</v>
       </c>
       <c r="C3" t="n">
-        <v>0.185935126661433</v>
+        <v>0.06962575577076313</v>
       </c>
       <c r="D3" t="n">
-        <v>-7.685102263641584</v>
+        <v>-7.719060471503303</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.4942623523935781</v>
+        <v>-0.9403823629269489</v>
       </c>
       <c r="F3" t="n">
-        <v>0.2642325247290501</v>
+        <v>0.0887674678201098</v>
       </c>
       <c r="G3" t="n">
-        <v>-2.056534362470479</v>
+        <v>-2.261472986053988</v>
       </c>
       <c r="H3" t="n">
-        <v>-2.569663161704924</v>
+        <v>-2.828885309098955</v>
       </c>
     </row>
     <row r="4">
@@ -514,25 +514,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2.145285387909215</v>
+        <v>2.183053147462237</v>
       </c>
       <c r="C4" t="n">
-        <v>0.9441303660461327</v>
+        <v>0.9010011207094546</v>
       </c>
       <c r="D4" t="n">
-        <v>-4.935315787765843</v>
+        <v>-4.647871499401919</v>
       </c>
       <c r="E4" t="n">
-        <v>0.3861605494553635</v>
+        <v>0.485893467275696</v>
       </c>
       <c r="F4" t="n">
-        <v>1.01051083402168</v>
+        <v>1.029752837070234</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.9326538364255732</v>
+        <v>-0.9379942863260402</v>
       </c>
       <c r="H4" t="n">
-        <v>-2.180691731084563</v>
+        <v>-1.921954054964888</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finalize plots & tables
</commit_message>
<xml_diff>
--- a/Tables/AAR_harris.xlsx
+++ b/Tables/AAR_harris.xlsx
@@ -486,25 +486,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.107004786128738</v>
+        <v>1.102762185566807</v>
       </c>
       <c r="C3" t="n">
-        <v>0.06962575577076313</v>
+        <v>0.06534335372761194</v>
       </c>
       <c r="D3" t="n">
-        <v>-7.719060471503303</v>
+        <v>-7.72528014984524</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.9403823629269489</v>
+        <v>-0.9490985384539019</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0887674678201098</v>
+        <v>0.09027056503920772</v>
       </c>
       <c r="G3" t="n">
-        <v>-2.261472986053988</v>
+        <v>-2.242361189394264</v>
       </c>
       <c r="H3" t="n">
-        <v>-2.828885309098955</v>
+        <v>-2.823510466904599</v>
       </c>
     </row>
     <row r="4">
@@ -514,25 +514,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2.183053147462237</v>
+        <v>2.177563842053711</v>
       </c>
       <c r="C4" t="n">
-        <v>0.9010011207094546</v>
+        <v>0.9043060068786674</v>
       </c>
       <c r="D4" t="n">
-        <v>-4.647871499401919</v>
+        <v>-4.611833258800136</v>
       </c>
       <c r="E4" t="n">
-        <v>0.485893467275696</v>
+        <v>0.4923639071080997</v>
       </c>
       <c r="F4" t="n">
-        <v>1.029752837070234</v>
+        <v>1.036119211930935</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.9379942863260402</v>
+        <v>-0.9456222154754571</v>
       </c>
       <c r="H4" t="n">
-        <v>-1.921954054964888</v>
+        <v>-1.945586252086026</v>
       </c>
     </row>
   </sheetData>

</xml_diff>